<commit_message>
fixed the issues for test_update_address test case
</commit_message>
<xml_diff>
--- a/data/web/address_data.xlsx
+++ b/data/web/address_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wealt\AI_Playwright_Python_Project\data\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7E7234-DBC4-44B1-B2DC-8742639B75FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B38C30D-D9DB-4A4C-832A-BD09D4D040C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,7 +81,7 @@
     <t>Shilpa Valley Road</t>
   </si>
   <si>
-    <t>ABCd</t>
+    <t>xyz</t>
   </si>
 </sst>
 </file>

</xml_diff>